<commit_message>
Fixing importing chartres DS
</commit_message>
<xml_diff>
--- a/src/main/resources/datasets/Import_Chartres.xlsx
+++ b/src/main/resources/datasets/Import_Chartres.xlsx
@@ -66,7 +66,7 @@
         <color indexed="11"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idt=th230</t>
+      <t>https://thesaurus.mom.fr/?idt=th258</t>
     </r>
   </si>
   <si>
@@ -938,7 +938,7 @@
         <color indexed="11"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230</t>
+      <t>https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258</t>
     </r>
   </si>
   <si>
@@ -988,7 +988,7 @@
         <color indexed="11"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230</t>
+      <t>https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258</t>
     </r>
   </si>
   <si>
@@ -3352,10 +3352,10 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="37.7891" style="1" customWidth="1"/>
+    <col min="1" max="1" width="37.8516" style="1" customWidth="1"/>
     <col min="2" max="2" width="54" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="46.1953" style="1" customWidth="1"/>
+    <col min="4" max="4" width="46.1719" style="1" customWidth="1"/>
     <col min="5" max="5" width="30" style="1" customWidth="1"/>
     <col min="6" max="16384" width="12.6719" style="1" customWidth="1"/>
   </cols>
@@ -3463,7 +3463,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" location="" tooltip="" display="admin@siamois.fr"/>
-    <hyperlink ref="E2" r:id="rId2" location="" tooltip="" display="https://thesaurus.mom.fr/?idt=th230"/>
+    <hyperlink ref="E2" r:id="rId2" location="" tooltip="" display="https://thesaurus.mom.fr/?idt=th258"/>
     <hyperlink ref="E3" r:id="rId3" location="" tooltip="" display="https://thesaurus.mom.fr/?idt=th240"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
@@ -30487,7 +30487,7 @@
     <col min="2" max="2" width="37.8516" style="40" customWidth="1"/>
     <col min="3" max="3" width="21.3516" style="40" customWidth="1"/>
     <col min="4" max="4" width="12.6719" style="40" customWidth="1"/>
-    <col min="5" max="5" width="115.367" style="40" customWidth="1"/>
+    <col min="5" max="5" width="115.352" style="40" customWidth="1"/>
     <col min="6" max="16384" width="12.6719" style="40" customWidth="1"/>
   </cols>
   <sheetData>
@@ -47323,26 +47323,26 @@
     <hyperlink ref="C58" r:id="rId151" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287629&amp;idt=th230"/>
     <hyperlink ref="C59" r:id="rId152" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287629&amp;idt=th230"/>
     <hyperlink ref="C60" r:id="rId153" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287629&amp;idt=th230"/>
-    <hyperlink ref="C61" r:id="rId154" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C62" r:id="rId155" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C63" r:id="rId156" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C64" r:id="rId157" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C65" r:id="rId158" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C66" r:id="rId159" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C67" r:id="rId160" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C68" r:id="rId161" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C69" r:id="rId162" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C70" r:id="rId163" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C71" r:id="rId164" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C72" r:id="rId165" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C73" r:id="rId166" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288312&amp;idt=th230"/>
-    <hyperlink ref="C74" r:id="rId167" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
-    <hyperlink ref="C75" r:id="rId168" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
-    <hyperlink ref="C76" r:id="rId169" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
-    <hyperlink ref="C77" r:id="rId170" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
-    <hyperlink ref="C78" r:id="rId171" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
-    <hyperlink ref="C79" r:id="rId172" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
-    <hyperlink ref="C80" r:id="rId173" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4288313&amp;idt=th230"/>
+    <hyperlink ref="C61" r:id="rId154" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C62" r:id="rId155" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C63" r:id="rId156" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C64" r:id="rId157" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C65" r:id="rId158" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C66" r:id="rId159" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C67" r:id="rId160" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C68" r:id="rId161" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C69" r:id="rId162" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C70" r:id="rId163" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C71" r:id="rId164" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C72" r:id="rId165" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C73" r:id="rId166" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289298&amp;idt=th258"/>
+    <hyperlink ref="C74" r:id="rId167" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
+    <hyperlink ref="C75" r:id="rId168" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
+    <hyperlink ref="C76" r:id="rId169" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
+    <hyperlink ref="C77" r:id="rId170" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
+    <hyperlink ref="C78" r:id="rId171" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
+    <hyperlink ref="C79" r:id="rId172" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
+    <hyperlink ref="C80" r:id="rId173" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4289299&amp;idt=th258"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>